<commit_message>
feat: add Odoo automation script, configuration, excel handler, and input datasets for testing
</commit_message>
<xml_diff>
--- a/Rencana/RENCANA.xlsx
+++ b/Rencana/RENCANA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python\odooCompressionTest\Rencana\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Septian Ferry\Dokumen\Project\odooCompressionTest\odooCompressionTest\Rencana\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B2A06D-1EDF-4427-B374-0676D48E9D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E1D6192-815F-4EAD-B1AE-DD0E6C2F6633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="84">
   <si>
     <t>Docket</t>
   </si>
@@ -105,37 +105,49 @@
     <t>Silinder 15 x 30 cm</t>
   </si>
   <si>
+    <t>Tidak</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/06-2026/01312</t>
+  </si>
+  <si>
+    <t>JALAN TOL AKSES PATIMBAN PAKET 4</t>
+  </si>
+  <si>
+    <t>WIKA-ADHI JO</t>
+  </si>
+  <si>
+    <t>CTB 4% NFA-0 NFA</t>
+  </si>
+  <si>
     <t>Belum_Test</t>
   </si>
   <si>
-    <t>Tidak</t>
-  </si>
-  <si>
-    <t>Patimban Port Development Project Package 6 : Container Terminal No.2 Construction</t>
-  </si>
-  <si>
-    <t>PENTA OCEAN-TOYO-RINKAI-PP-WIKA-JAKON CONSORTIUM</t>
-  </si>
-  <si>
-    <t>Class A-2 NFA</t>
-  </si>
-  <si>
-    <t>JALAN TOL AKSES PATIMBAN PAKET 4</t>
-  </si>
-  <si>
-    <t>WIKA-ADHI JO</t>
-  </si>
-  <si>
-    <t>SO/DIR2/DV2-4/09-2026/02138</t>
-  </si>
-  <si>
-    <t>Class D-1 NFA</t>
-  </si>
-  <si>
-    <t>WIKA - ADHI JO / DS 1.1 PS.18 / CLASS D-1 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09028</t>
+    <t>Pembangunan Jalan Tol Akses Patimban Paket 3</t>
+  </si>
+  <si>
+    <t>HUTAMA KARYA - JAYA KONSTRUKSI JOINT OPERATION</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/09-2026/02508</t>
+  </si>
+  <si>
+    <t>CTB 3 %-0 NFA</t>
+  </si>
+  <si>
+    <t>Class E-1 NFA</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/10-2026/02610</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/05-2026/01082</t>
+  </si>
+  <si>
+    <t>Class C-1 NFA</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10340</t>
   </si>
   <si>
     <t>SO/DIR2/DV2-4/05-2026/01028</t>
@@ -150,112 +162,130 @@
     <t>Fc-30 NFA</t>
   </si>
   <si>
-    <t>PP - TOL PTB / ISIAN PANCANG P2 B7 STA 20+091 / FC 30 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09029</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09040</t>
-  </si>
-  <si>
-    <t>SO/DIR2/DV2-4/08-2026/01880</t>
-  </si>
-  <si>
-    <t>K-125 NFA</t>
-  </si>
-  <si>
-    <t>PP - TOL PTB / LC PLAT INJAK BOX CULVERT STA 16+060 / K 125 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09036</t>
-  </si>
-  <si>
-    <t>SO/DIR2/DV2-4/07-2026/01764</t>
-  </si>
-  <si>
-    <t>Class G NFA-3 NFA</t>
-  </si>
-  <si>
-    <t>PTRPWJ / PC SLAB PAV - / CLASS G-3 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09041</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09043</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09042</t>
-  </si>
-  <si>
-    <t>SO/DIR2/DV2-4/07-2026/01560</t>
-  </si>
-  <si>
-    <t>PTRPWJ / RIGID PAV - 17825 / CLASS A-2 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09045</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09046</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09024</t>
-  </si>
-  <si>
-    <t>SO/DIR2/DV2-4/06-2026/01312</t>
-  </si>
-  <si>
-    <t>CTB 4% NFA-0 NFA</t>
-  </si>
-  <si>
-    <t>WIKA - ADHI JO / RAMP 6 / CTB 4% / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09027</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09032</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/08-2026/09035</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09963</t>
-  </si>
-  <si>
-    <t>PP - TOL PTB / HEADWALL P1 B7 STA 20+000 / FC 30 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09965</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09940</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09956</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09942</t>
-  </si>
-  <si>
-    <t>WIKA - ADHI JO / STA 34+887 R1 / CTB 4% / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09945</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09950</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09953</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09957</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/09961</t>
+    <t>PP - TOL PTB / PILECAPE P2 STG.3 B.7 STA 20+000 / FC 30 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10297</t>
+  </si>
+  <si>
+    <t>WIKA - ADHI JO / CROSS DRAIN RAMP AKSES / CLASS C-1 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10315</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10273</t>
+  </si>
+  <si>
+    <t>WIKA - ADHI JO / STA 35+400 L2 / CTB 4% / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10280</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10285</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10296</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10304</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10310</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10313</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10317</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11240</t>
+  </si>
+  <si>
+    <t>SO/DV2-4/10-2026/01588</t>
+  </si>
+  <si>
+    <t>Peningkatan Jl. Kab. Karang Anyar - Compreng</t>
+  </si>
+  <si>
+    <t>CV ALPIN ALGANI</t>
+  </si>
+  <si>
+    <t>Fc-10 FA</t>
+  </si>
+  <si>
+    <t>CV ALPIN ALGANI / FC 10 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11245</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11235</t>
+  </si>
+  <si>
+    <t>HK - JAKON JO / STA 29+925 - STA 30+050 / CTB 3% / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11241</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11249</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11251</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11257</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/07-2026/01540</t>
+  </si>
+  <si>
+    <t>GA Warehouse Building of Vinfast Phase 2 Project</t>
+  </si>
+  <si>
+    <t>PT. MURINDA IRON STEEL</t>
+  </si>
+  <si>
+    <t>K-400 NFA</t>
+  </si>
+  <si>
+    <t>MURINDA / K 400 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11259</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11256</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/10-2026/02628</t>
+  </si>
+  <si>
+    <t>Cv.Sebelas Sodara</t>
+  </si>
+  <si>
+    <t>PT. SULTAN PANDAWA GROUP</t>
+  </si>
+  <si>
+    <t>SULTAN PANDAWA / FC 10 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11236</t>
+  </si>
+  <si>
+    <t>WIKA - ADHI JO / LC MAINROAD STA 35+315 - STA 35+351 / CLASS E / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11246</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11253</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11255</t>
   </si>
 </sst>
 </file>
@@ -324,8 +354,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
@@ -335,9 +366,10 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 94" xfId="1" xr:uid="{74C35DD4-AD32-431F-A3CB-06EF28F4517C}"/>
+    <cellStyle name="Normal 95" xfId="2" xr:uid="{642106DB-F03E-45E3-9C43-12A12BC120C6}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -639,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -655,7 +687,7 @@
     <col min="17" max="22" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -725,25 +757,25 @@
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
       <c r="H2" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I2">
         <v>28</v>
@@ -758,13 +790,13 @@
         <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -787,25 +819,25 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G3">
         <v>4</v>
       </c>
       <c r="H3" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I3">
         <v>28</v>
@@ -820,13 +852,13 @@
         <v>0</v>
       </c>
       <c r="N3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -849,25 +881,25 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
         <v>36</v>
-      </c>
-      <c r="F4" t="s">
-        <v>37</v>
       </c>
       <c r="G4">
         <v>3</v>
       </c>
       <c r="H4" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I4">
         <v>28</v>
@@ -882,13 +914,13 @@
         <v>0</v>
       </c>
       <c r="N4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -911,25 +943,25 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>36</v>
-      </c>
-      <c r="F5" t="s">
-        <v>37</v>
       </c>
       <c r="G5">
         <v>4</v>
       </c>
       <c r="H5" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I5">
         <v>28</v>
@@ -944,13 +976,13 @@
         <v>0</v>
       </c>
       <c r="N5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P5" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -973,25 +1005,25 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
         <v>36</v>
-      </c>
-      <c r="F6" t="s">
-        <v>42</v>
       </c>
       <c r="G6">
         <v>3</v>
       </c>
       <c r="H6" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I6">
         <v>28</v>
@@ -1006,13 +1038,13 @@
         <v>0</v>
       </c>
       <c r="N6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -1035,25 +1067,25 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
         <v>36</v>
-      </c>
-      <c r="F7" t="s">
-        <v>42</v>
       </c>
       <c r="G7">
         <v>4</v>
       </c>
       <c r="H7" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I7">
         <v>28</v>
@@ -1068,13 +1100,13 @@
         <v>0</v>
       </c>
       <c r="N7" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -1097,10 +1129,10 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
         <v>25</v>
@@ -1109,13 +1141,13 @@
         <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G8">
         <v>3</v>
       </c>
       <c r="H8" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I8">
         <v>28</v>
@@ -1130,10 +1162,10 @@
         <v>0</v>
       </c>
       <c r="N8" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P8" t="s">
         <v>47</v>
@@ -1159,10 +1191,10 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
@@ -1171,13 +1203,13 @@
         <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G9">
         <v>4</v>
       </c>
       <c r="H9" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I9">
         <v>28</v>
@@ -1192,10 +1224,10 @@
         <v>0</v>
       </c>
       <c r="N9" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P9" t="s">
         <v>47</v>
@@ -1224,7 +1256,7 @@
         <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
         <v>25</v>
@@ -1233,13 +1265,13 @@
         <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G10">
         <v>3</v>
       </c>
       <c r="H10" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I10">
         <v>28</v>
@@ -1254,10 +1286,10 @@
         <v>0</v>
       </c>
       <c r="N10" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P10" t="s">
         <v>47</v>
@@ -1286,7 +1318,7 @@
         <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
         <v>25</v>
@@ -1295,13 +1327,13 @@
         <v>26</v>
       </c>
       <c r="F11" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G11">
         <v>4</v>
       </c>
       <c r="H11" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I11">
         <v>28</v>
@@ -1316,10 +1348,10 @@
         <v>0</v>
       </c>
       <c r="N11" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P11" t="s">
         <v>47</v>
@@ -1348,7 +1380,7 @@
         <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
         <v>25</v>
@@ -1357,13 +1389,13 @@
         <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G12">
         <v>3</v>
       </c>
       <c r="H12" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I12">
         <v>28</v>
@@ -1378,10 +1410,10 @@
         <v>0</v>
       </c>
       <c r="N12" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P12" t="s">
         <v>47</v>
@@ -1410,7 +1442,7 @@
         <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="D13" t="s">
         <v>25</v>
@@ -1419,13 +1451,13 @@
         <v>26</v>
       </c>
       <c r="F13" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G13">
         <v>4</v>
       </c>
       <c r="H13" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I13">
         <v>28</v>
@@ -1440,10 +1472,10 @@
         <v>0</v>
       </c>
       <c r="N13" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P13" t="s">
         <v>47</v>
@@ -1472,7 +1504,7 @@
         <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D14" t="s">
         <v>25</v>
@@ -1487,7 +1519,7 @@
         <v>3</v>
       </c>
       <c r="H14" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I14">
         <v>28</v>
@@ -1502,13 +1534,13 @@
         <v>0</v>
       </c>
       <c r="N14" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P14" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1534,7 +1566,7 @@
         <v>50</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D15" t="s">
         <v>25</v>
@@ -1549,7 +1581,7 @@
         <v>4</v>
       </c>
       <c r="H15" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I15">
         <v>28</v>
@@ -1564,13 +1596,13 @@
         <v>0</v>
       </c>
       <c r="N15" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P15" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1593,10 +1625,10 @@
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D16" t="s">
         <v>25</v>
@@ -1611,7 +1643,7 @@
         <v>3</v>
       </c>
       <c r="H16" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I16">
         <v>28</v>
@@ -1626,13 +1658,13 @@
         <v>0</v>
       </c>
       <c r="N16" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P16" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1655,10 +1687,10 @@
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D17" t="s">
         <v>25</v>
@@ -1673,7 +1705,7 @@
         <v>4</v>
       </c>
       <c r="H17" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I17">
         <v>28</v>
@@ -1688,13 +1720,13 @@
         <v>0</v>
       </c>
       <c r="N17" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P17" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="Q17" t="b">
         <v>0</v>
@@ -1717,10 +1749,10 @@
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D18" t="s">
         <v>25</v>
@@ -1735,7 +1767,7 @@
         <v>3</v>
       </c>
       <c r="H18" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I18">
         <v>28</v>
@@ -1750,13 +1782,13 @@
         <v>0</v>
       </c>
       <c r="N18" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P18" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1779,10 +1811,10 @@
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
@@ -1797,7 +1829,7 @@
         <v>4</v>
       </c>
       <c r="H19" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I19">
         <v>28</v>
@@ -1812,13 +1844,13 @@
         <v>0</v>
       </c>
       <c r="N19" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P19" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="Q19" t="b">
         <v>0</v>
@@ -1841,25 +1873,25 @@
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F20" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="G20">
         <v>3</v>
       </c>
       <c r="H20" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I20">
         <v>28</v>
@@ -1874,13 +1906,13 @@
         <v>0</v>
       </c>
       <c r="N20" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P20" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="Q20" t="b">
         <v>0</v>
@@ -1903,25 +1935,25 @@
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="G21">
         <v>4</v>
       </c>
       <c r="H21" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I21">
         <v>28</v>
@@ -1936,13 +1968,13 @@
         <v>0</v>
       </c>
       <c r="N21" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P21" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="Q21" t="b">
         <v>0</v>
@@ -1965,25 +1997,25 @@
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F22" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="G22">
         <v>3</v>
       </c>
       <c r="H22" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I22">
         <v>28</v>
@@ -1998,13 +2030,13 @@
         <v>0</v>
       </c>
       <c r="N22" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P22" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="Q22" t="b">
         <v>0</v>
@@ -2027,25 +2059,25 @@
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F23" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="G23">
         <v>4</v>
       </c>
       <c r="H23" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I23">
         <v>28</v>
@@ -2060,13 +2092,13 @@
         <v>0</v>
       </c>
       <c r="N23" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P23" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="Q23" t="b">
         <v>0</v>
@@ -2089,46 +2121,46 @@
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B24" t="s">
         <v>56</v>
       </c>
       <c r="D24" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="E24" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F24" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H24" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I24">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J24" t="s">
         <v>22</v>
       </c>
       <c r="K24">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M24">
         <v>0</v>
       </c>
       <c r="N24" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P24" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q24" t="b">
         <v>0</v>
@@ -2151,46 +2183,46 @@
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B25" t="s">
         <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="E25" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F25" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H25" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I25">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J25" t="s">
         <v>22</v>
       </c>
       <c r="K25">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M25">
         <v>0</v>
       </c>
       <c r="N25" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q25" t="b">
         <v>0</v>
@@ -2219,40 +2251,40 @@
         <v>56</v>
       </c>
       <c r="D26" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="E26" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H26" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I26">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J26" t="s">
         <v>22</v>
       </c>
       <c r="K26">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M26">
         <v>0</v>
       </c>
       <c r="N26" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q26" t="b">
         <v>0</v>
@@ -2281,40 +2313,40 @@
         <v>56</v>
       </c>
       <c r="D27" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="E27" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="F27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H27" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I27">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="J27" t="s">
         <v>22</v>
       </c>
       <c r="K27">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M27">
         <v>0</v>
       </c>
       <c r="N27" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q27" t="b">
         <v>0</v>
@@ -2340,22 +2372,22 @@
         <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D28" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E28" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F28" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G28">
         <v>1</v>
       </c>
       <c r="H28" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I28">
         <v>7</v>
@@ -2370,10 +2402,10 @@
         <v>0</v>
       </c>
       <c r="N28" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P28" t="s">
         <v>63</v>
@@ -2402,22 +2434,22 @@
         <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D29" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E29" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F29" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G29">
         <v>2</v>
       </c>
       <c r="H29" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I29">
         <v>7</v>
@@ -2432,10 +2464,10 @@
         <v>0</v>
       </c>
       <c r="N29" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P29" t="s">
         <v>63</v>
@@ -2464,22 +2496,22 @@
         <v>64</v>
       </c>
       <c r="B30" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D30" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E30" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F30" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G30">
         <v>1</v>
       </c>
       <c r="H30" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I30">
         <v>7</v>
@@ -2494,10 +2526,10 @@
         <v>0</v>
       </c>
       <c r="N30" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O30" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P30" t="s">
         <v>63</v>
@@ -2526,22 +2558,22 @@
         <v>64</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D31" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E31" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F31" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G31">
         <v>2</v>
       </c>
       <c r="H31" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I31">
         <v>7</v>
@@ -2556,10 +2588,10 @@
         <v>0</v>
       </c>
       <c r="N31" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P31" t="s">
         <v>63</v>
@@ -2588,22 +2620,22 @@
         <v>65</v>
       </c>
       <c r="B32" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E32" t="s">
         <v>30</v>
       </c>
-      <c r="D32" t="s">
-        <v>28</v>
-      </c>
-      <c r="E32" t="s">
-        <v>29</v>
-      </c>
       <c r="F32" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
       <c r="H32" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I32">
         <v>7</v>
@@ -2618,13 +2650,13 @@
         <v>0</v>
       </c>
       <c r="N32" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P32" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="Q32" t="b">
         <v>0</v>
@@ -2650,22 +2682,22 @@
         <v>65</v>
       </c>
       <c r="B33" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33" t="s">
         <v>30</v>
       </c>
-      <c r="D33" t="s">
-        <v>28</v>
-      </c>
-      <c r="E33" t="s">
-        <v>29</v>
-      </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G33">
         <v>2</v>
       </c>
       <c r="H33" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I33">
         <v>7</v>
@@ -2680,13 +2712,13 @@
         <v>0</v>
       </c>
       <c r="N33" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O33" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P33" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="Q33" t="b">
         <v>0</v>
@@ -2712,22 +2744,22 @@
         <v>66</v>
       </c>
       <c r="B34" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" t="s">
+        <v>29</v>
+      </c>
+      <c r="E34" t="s">
         <v>30</v>
       </c>
-      <c r="D34" t="s">
-        <v>28</v>
-      </c>
-      <c r="E34" t="s">
-        <v>29</v>
-      </c>
       <c r="F34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
       <c r="H34" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I34">
         <v>7</v>
@@ -2742,13 +2774,13 @@
         <v>0</v>
       </c>
       <c r="N34" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O34" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P34" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="Q34" t="b">
         <v>0</v>
@@ -2774,22 +2806,22 @@
         <v>66</v>
       </c>
       <c r="B35" t="s">
+        <v>31</v>
+      </c>
+      <c r="D35" t="s">
+        <v>29</v>
+      </c>
+      <c r="E35" t="s">
         <v>30</v>
       </c>
-      <c r="D35" t="s">
-        <v>28</v>
-      </c>
-      <c r="E35" t="s">
-        <v>29</v>
-      </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G35">
         <v>2</v>
       </c>
       <c r="H35" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I35">
         <v>7</v>
@@ -2804,13 +2836,13 @@
         <v>0</v>
       </c>
       <c r="N35" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P35" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="Q35" t="b">
         <v>0</v>
@@ -2836,22 +2868,22 @@
         <v>67</v>
       </c>
       <c r="B36" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="D36" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="E36" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F36" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="G36">
         <v>1</v>
       </c>
       <c r="H36" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I36">
         <v>7</v>
@@ -2866,13 +2898,13 @@
         <v>0</v>
       </c>
       <c r="N36" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O36" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P36" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="Q36" t="b">
         <v>0</v>
@@ -2898,22 +2930,22 @@
         <v>67</v>
       </c>
       <c r="B37" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="D37" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="E37" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F37" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="G37">
         <v>2</v>
       </c>
       <c r="H37" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I37">
         <v>7</v>
@@ -2928,13 +2960,13 @@
         <v>0</v>
       </c>
       <c r="N37" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P37" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="Q37" t="b">
         <v>0</v>
@@ -2957,25 +2989,25 @@
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" t="s">
+        <v>68</v>
+      </c>
+      <c r="D38" t="s">
         <v>69</v>
       </c>
-      <c r="B38" t="s">
-        <v>56</v>
-      </c>
-      <c r="D38" t="s">
-        <v>28</v>
-      </c>
       <c r="E38" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F38" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="G38">
         <v>1</v>
       </c>
       <c r="H38" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I38">
         <v>7</v>
@@ -2990,13 +3022,13 @@
         <v>0</v>
       </c>
       <c r="N38" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P38" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="Q38" t="b">
         <v>0</v>
@@ -3019,25 +3051,25 @@
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>73</v>
+      </c>
+      <c r="B39" t="s">
+        <v>68</v>
+      </c>
+      <c r="D39" t="s">
         <v>69</v>
       </c>
-      <c r="B39" t="s">
-        <v>56</v>
-      </c>
-      <c r="D39" t="s">
-        <v>28</v>
-      </c>
       <c r="E39" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="F39" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="G39">
         <v>2</v>
       </c>
       <c r="H39" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I39">
         <v>7</v>
@@ -3052,13 +3084,13 @@
         <v>0</v>
       </c>
       <c r="N39" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P39" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="Q39" t="b">
         <v>0</v>
@@ -3081,25 +3113,25 @@
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B40" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="D40" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="E40" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="F40" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G40">
         <v>1</v>
       </c>
       <c r="H40" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I40">
         <v>7</v>
@@ -3114,13 +3146,13 @@
         <v>0</v>
       </c>
       <c r="N40" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P40" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="Q40" t="b">
         <v>0</v>
@@ -3143,25 +3175,25 @@
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="D41" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="E41" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="F41" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G41">
         <v>2</v>
       </c>
       <c r="H41" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I41">
         <v>7</v>
@@ -3176,13 +3208,13 @@
         <v>0</v>
       </c>
       <c r="N41" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O41" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P41" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="Q41" t="b">
         <v>0</v>
@@ -3205,25 +3237,25 @@
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B42" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="D42" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E42" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F42" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="G42">
         <v>1</v>
       </c>
       <c r="H42" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I42">
         <v>7</v>
@@ -3238,13 +3270,13 @@
         <v>0</v>
       </c>
       <c r="N42" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P42" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="Q42" t="b">
         <v>0</v>
@@ -3267,25 +3299,25 @@
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="B43" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="D43" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E43" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F43" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="G43">
         <v>2</v>
       </c>
       <c r="H43" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I43">
         <v>7</v>
@@ -3300,13 +3332,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P43" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="Q43" t="b">
         <v>0</v>
@@ -3329,25 +3361,25 @@
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="B44" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E44" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F44" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="G44">
         <v>1</v>
       </c>
       <c r="H44" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I44">
         <v>7</v>
@@ -3362,13 +3394,13 @@
         <v>0</v>
       </c>
       <c r="N44" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O44" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P44" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="Q44" t="b">
         <v>0</v>
@@ -3391,25 +3423,25 @@
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="D45" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E45" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F45" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="G45">
         <v>2</v>
       </c>
       <c r="H45" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I45">
         <v>7</v>
@@ -3424,13 +3456,13 @@
         <v>0</v>
       </c>
       <c r="N45" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O45" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P45" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="Q45" t="b">
         <v>0</v>
@@ -3453,25 +3485,25 @@
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="B46" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="D46" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E46" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F46" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="G46">
         <v>1</v>
       </c>
       <c r="H46" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I46">
         <v>7</v>
@@ -3486,13 +3518,13 @@
         <v>0</v>
       </c>
       <c r="N46" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O46" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P46" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="Q46" t="b">
         <v>0</v>
@@ -3515,25 +3547,25 @@
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="D47" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E47" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F47" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="G47">
         <v>2</v>
       </c>
       <c r="H47" s="2">
-        <v>46280</v>
+        <v>46308</v>
       </c>
       <c r="I47">
         <v>7</v>
@@ -3548,13 +3580,13 @@
         <v>0</v>
       </c>
       <c r="N47" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="O47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="P47" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="Q47" t="b">
         <v>0</v>
@@ -3572,6 +3604,130 @@
         <v>0</v>
       </c>
       <c r="V47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>83</v>
+      </c>
+      <c r="B48" t="s">
+        <v>34</v>
+      </c>
+      <c r="D48" t="s">
+        <v>25</v>
+      </c>
+      <c r="E48" t="s">
+        <v>26</v>
+      </c>
+      <c r="F48" t="s">
+        <v>33</v>
+      </c>
+      <c r="G48">
+        <v>1</v>
+      </c>
+      <c r="H48" s="2">
+        <v>46308</v>
+      </c>
+      <c r="I48">
+        <v>7</v>
+      </c>
+      <c r="J48" t="s">
+        <v>22</v>
+      </c>
+      <c r="K48">
+        <v>65</v>
+      </c>
+      <c r="M48">
+        <v>0</v>
+      </c>
+      <c r="N48" t="s">
+        <v>28</v>
+      </c>
+      <c r="O48" t="s">
+        <v>23</v>
+      </c>
+      <c r="P48" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q48" t="b">
+        <v>0</v>
+      </c>
+      <c r="R48">
+        <v>0</v>
+      </c>
+      <c r="S48">
+        <v>0</v>
+      </c>
+      <c r="T48">
+        <v>0</v>
+      </c>
+      <c r="U48">
+        <v>0</v>
+      </c>
+      <c r="V48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>83</v>
+      </c>
+      <c r="B49" t="s">
+        <v>34</v>
+      </c>
+      <c r="D49" t="s">
+        <v>25</v>
+      </c>
+      <c r="E49" t="s">
+        <v>26</v>
+      </c>
+      <c r="F49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49">
+        <v>2</v>
+      </c>
+      <c r="H49" s="2">
+        <v>46308</v>
+      </c>
+      <c r="I49">
+        <v>7</v>
+      </c>
+      <c r="J49" t="s">
+        <v>22</v>
+      </c>
+      <c r="K49">
+        <v>65</v>
+      </c>
+      <c r="M49">
+        <v>0</v>
+      </c>
+      <c r="N49" t="s">
+        <v>28</v>
+      </c>
+      <c r="O49" t="s">
+        <v>23</v>
+      </c>
+      <c r="P49" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q49" t="b">
+        <v>0</v>
+      </c>
+      <c r="R49">
+        <v>0</v>
+      </c>
+      <c r="S49">
+        <v>0</v>
+      </c>
+      <c r="T49">
+        <v>0</v>
+      </c>
+      <c r="U49">
+        <v>0</v>
+      </c>
+      <c r="V49">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add core modules, UI components, and installer configuration for compression test application
</commit_message>
<xml_diff>
--- a/Rencana/RENCANA.xlsx
+++ b/Rencana/RENCANA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Septian Ferry\Dokumen\Project\odooCompressionTest\odooCompressionTest\Rencana\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A9E4CF-07A5-4DA2-8E40-EA1F834558BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5015613-B712-4B4D-9C5C-0D9DFE461B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="84">
   <si>
     <t>Docket</t>
   </si>
@@ -117,40 +117,175 @@
     <t>HUTAMA KARYA - JAYA KONSTRUKSI JOINT OPERATION</t>
   </si>
   <si>
-    <t>DOCKET/PTB/09-2026/10395</t>
-  </si>
-  <si>
     <t>SO/DIR2/DV2-4/07-2026/01578</t>
   </si>
   <si>
+    <t>JALAN TOL AKSES PATIMBAN PAKET 4</t>
+  </si>
+  <si>
+    <t>WIKA-ADHI JO</t>
+  </si>
+  <si>
+    <t>Class D-1 NFA</t>
+  </si>
+  <si>
     <t>Class B-1 FA</t>
   </si>
   <si>
-    <t>HK - JAKON JO / DECKSLAB PE2 - AE2 BRIDGE 17 STA 30+700 / CLASS B-1 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/10397</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/10401</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/10404</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/10407</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/10409</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/10393</t>
-  </si>
-  <si>
-    <t>HK - JAKON JO / HALFSLAB S1 (7 UNIT) PS.14 STA 31+000 / CLASS B-1 / AD PTB</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/09-2026/10394</t>
+    <t>CTB 3 %-0 NFA</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/09-2026/02374</t>
+  </si>
+  <si>
+    <t>Beam 15 x 15 x 60 cm</t>
+  </si>
+  <si>
+    <t>PT. SULTAN PANDAWA GROUP</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/05-2026/01082</t>
+  </si>
+  <si>
+    <t>Class C-1 NFA</t>
+  </si>
+  <si>
+    <t>Fs-35 NFA</t>
+  </si>
+  <si>
+    <t>RIZKUNA BAROQAH</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10790</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-2/09-2026/01100</t>
+  </si>
+  <si>
+    <t>Pondasi PJU</t>
+  </si>
+  <si>
+    <t>COMPLUS SISTEM SOLUSI</t>
+  </si>
+  <si>
+    <t>K-250 FA</t>
+  </si>
+  <si>
+    <t>22-10-2026 00:00:00</t>
+  </si>
+  <si>
+    <t>COMPLUS SISTEM SOLUSI / K 250 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10798</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10803</t>
+  </si>
+  <si>
+    <t>HK - JAKON JO / BARRIER PE2 - AE2 MEDIAN &amp; TEPI BRIDGE 17 STA 30+600 / CLASS B-1 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10808</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10812</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10792</t>
+  </si>
+  <si>
+    <t>Class E-1 FA</t>
+  </si>
+  <si>
+    <t>HK - JAKON JO / LC DETOUR OP.6 STA 32+048 / CLASS E / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10793</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/09-2026/10789</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/08-2026/01784</t>
+  </si>
+  <si>
+    <t>PT Tesco Indomaritim</t>
+  </si>
+  <si>
+    <t>PT. TESCO INDOMARITIM</t>
+  </si>
+  <si>
+    <t>K-350 NFA</t>
+  </si>
+  <si>
+    <t>TESCO INDOMARITIM / K 350 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11612</t>
+  </si>
+  <si>
+    <t>HK - JAKON JO / APPROACH SLAB A18 - P1 GRID A PS.15 / CLASS B-1 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11614</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11609</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/10-2026/02702</t>
+  </si>
+  <si>
+    <t>HK - JAKON JO / STA 29+537,5 - STA 29+650 L1 / CTB 3% / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11618</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11620</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11628</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/10-2026/02720</t>
+  </si>
+  <si>
+    <t>CV NAIRA GHAISANI</t>
+  </si>
+  <si>
+    <t>SULTAN PANDAWA / CV NAIRA GHAISANI / FS 38 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11630</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11627</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/10-2026/02676</t>
+  </si>
+  <si>
+    <t>SULTAN PANDAWA / RIZKUNA BAROQAH / FS 35 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11629</t>
+  </si>
+  <si>
+    <t>SO/DIR2/DV2-4/10-2026/02680</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11615</t>
+  </si>
+  <si>
+    <t>WIKA - ADHI JO / DS 1.2 STA 35+575 / CLASS D-1 / AD PTB</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/10-2026/11624</t>
+  </si>
+  <si>
+    <t>WIKA - ADHI JO / DS 3.3 STA 35+025 / CLASS C-1 / AD PTB</t>
   </si>
 </sst>
 </file>
@@ -224,12 +359,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V75"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.7109375" customWidth="1"/>
@@ -622,25 +756,25 @@
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
-      <c r="H2" s="2">
-        <v>46309</v>
+      <c r="H2" t="s">
+        <v>45</v>
       </c>
       <c r="I2">
         <v>28</v>
@@ -661,7 +795,7 @@
         <v>23</v>
       </c>
       <c r="P2" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="Q2" t="b">
         <v>0</v>
@@ -684,25 +818,25 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G3">
         <v>4</v>
       </c>
-      <c r="H3" s="2">
-        <v>46309</v>
+      <c r="H3" t="s">
+        <v>45</v>
       </c>
       <c r="I3">
         <v>28</v>
@@ -723,7 +857,7 @@
         <v>23</v>
       </c>
       <c r="P3" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="Q3" t="b">
         <v>0</v>
@@ -746,25 +880,25 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G4">
         <v>3</v>
       </c>
-      <c r="H4" s="2">
-        <v>46309</v>
+      <c r="H4" t="s">
+        <v>45</v>
       </c>
       <c r="I4">
         <v>28</v>
@@ -785,7 +919,7 @@
         <v>23</v>
       </c>
       <c r="P4" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
@@ -808,25 +942,25 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G5">
         <v>4</v>
       </c>
-      <c r="H5" s="2">
-        <v>46309</v>
+      <c r="H5" t="s">
+        <v>45</v>
       </c>
       <c r="I5">
         <v>28</v>
@@ -847,7 +981,7 @@
         <v>23</v>
       </c>
       <c r="P5" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
@@ -870,10 +1004,10 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
         <v>25</v>
@@ -882,13 +1016,13 @@
         <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6">
         <v>3</v>
       </c>
-      <c r="H6" s="2">
-        <v>46309</v>
+      <c r="H6" t="s">
+        <v>45</v>
       </c>
       <c r="I6">
         <v>28</v>
@@ -909,7 +1043,7 @@
         <v>23</v>
       </c>
       <c r="P6" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="Q6" t="b">
         <v>0</v>
@@ -932,10 +1066,10 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
         <v>25</v>
@@ -944,13 +1078,13 @@
         <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G7">
         <v>4</v>
       </c>
-      <c r="H7" s="2">
-        <v>46309</v>
+      <c r="H7" t="s">
+        <v>45</v>
       </c>
       <c r="I7">
         <v>28</v>
@@ -971,7 +1105,7 @@
         <v>23</v>
       </c>
       <c r="P7" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="Q7" t="b">
         <v>0</v>
@@ -994,10 +1128,10 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D8" t="s">
         <v>25</v>
@@ -1006,13 +1140,13 @@
         <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G8">
         <v>3</v>
       </c>
-      <c r="H8" s="2">
-        <v>46309</v>
+      <c r="H8" t="s">
+        <v>45</v>
       </c>
       <c r="I8">
         <v>28</v>
@@ -1033,7 +1167,7 @@
         <v>23</v>
       </c>
       <c r="P8" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1056,10 +1190,10 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
         <v>25</v>
@@ -1068,13 +1202,13 @@
         <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9">
         <v>4</v>
       </c>
-      <c r="H9" s="2">
-        <v>46309</v>
+      <c r="H9" t="s">
+        <v>45</v>
       </c>
       <c r="I9">
         <v>28</v>
@@ -1095,7 +1229,7 @@
         <v>23</v>
       </c>
       <c r="P9" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1118,10 +1252,10 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
         <v>25</v>
@@ -1130,13 +1264,13 @@
         <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10">
         <v>3</v>
       </c>
-      <c r="H10" s="2">
-        <v>46309</v>
+      <c r="H10" t="s">
+        <v>45</v>
       </c>
       <c r="I10">
         <v>28</v>
@@ -1157,7 +1291,7 @@
         <v>23</v>
       </c>
       <c r="P10" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="Q10" t="b">
         <v>0</v>
@@ -1180,10 +1314,10 @@
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
         <v>25</v>
@@ -1192,13 +1326,13 @@
         <v>26</v>
       </c>
       <c r="F11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G11">
         <v>4</v>
       </c>
-      <c r="H11" s="2">
-        <v>46309</v>
+      <c r="H11" t="s">
+        <v>45</v>
       </c>
       <c r="I11">
         <v>28</v>
@@ -1219,7 +1353,7 @@
         <v>23</v>
       </c>
       <c r="P11" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="Q11" t="b">
         <v>0</v>
@@ -1242,10 +1376,10 @@
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
         <v>25</v>
@@ -1254,13 +1388,13 @@
         <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="G12">
         <v>3</v>
       </c>
-      <c r="H12" s="2">
-        <v>46309</v>
+      <c r="H12" t="s">
+        <v>45</v>
       </c>
       <c r="I12">
         <v>28</v>
@@ -1281,7 +1415,7 @@
         <v>23</v>
       </c>
       <c r="P12" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="Q12" t="b">
         <v>0</v>
@@ -1304,10 +1438,10 @@
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
         <v>25</v>
@@ -1316,13 +1450,13 @@
         <v>26</v>
       </c>
       <c r="F13" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="G13">
         <v>4</v>
       </c>
-      <c r="H13" s="2">
-        <v>46309</v>
+      <c r="H13" t="s">
+        <v>45</v>
       </c>
       <c r="I13">
         <v>28</v>
@@ -1343,7 +1477,7 @@
         <v>23</v>
       </c>
       <c r="P13" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1366,10 +1500,10 @@
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D14" t="s">
         <v>25</v>
@@ -1378,13 +1512,13 @@
         <v>26</v>
       </c>
       <c r="F14" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="G14">
         <v>3</v>
       </c>
-      <c r="H14" s="2">
-        <v>46309</v>
+      <c r="H14" t="s">
+        <v>45</v>
       </c>
       <c r="I14">
         <v>28</v>
@@ -1405,7 +1539,7 @@
         <v>23</v>
       </c>
       <c r="P14" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1428,10 +1562,10 @@
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
         <v>25</v>
@@ -1440,13 +1574,13 @@
         <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="G15">
         <v>4</v>
       </c>
-      <c r="H15" s="2">
-        <v>46309</v>
+      <c r="H15" t="s">
+        <v>45</v>
       </c>
       <c r="I15">
         <v>28</v>
@@ -1467,7 +1601,7 @@
         <v>23</v>
       </c>
       <c r="P15" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="Q15" t="b">
         <v>0</v>
@@ -1490,25 +1624,25 @@
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="E16" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="F16" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="G16">
         <v>3</v>
       </c>
-      <c r="H16" s="2">
-        <v>46309</v>
+      <c r="H16" t="s">
+        <v>45</v>
       </c>
       <c r="I16">
         <v>28</v>
@@ -1529,7 +1663,7 @@
         <v>23</v>
       </c>
       <c r="P16" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="Q16" t="b">
         <v>0</v>
@@ -1552,25 +1686,25 @@
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="E17" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="F17" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="G17">
         <v>4</v>
       </c>
-      <c r="H17" s="2">
-        <v>46309</v>
+      <c r="H17" t="s">
+        <v>45</v>
       </c>
       <c r="I17">
         <v>28</v>
@@ -1591,200 +1725,1514 @@
         <v>23</v>
       </c>
       <c r="P17" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q17" t="b">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18" t="s">
+        <v>45</v>
+      </c>
+      <c r="I18">
+        <v>7</v>
+      </c>
+      <c r="J18" t="s">
+        <v>22</v>
+      </c>
+      <c r="K18">
+        <v>65</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18" t="s">
+        <v>24</v>
+      </c>
+      <c r="O18" t="s">
+        <v>23</v>
+      </c>
+      <c r="P18" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q18" t="b">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19" t="s">
+        <v>45</v>
+      </c>
+      <c r="I19">
+        <v>7</v>
+      </c>
+      <c r="J19" t="s">
+        <v>22</v>
+      </c>
+      <c r="K19">
+        <v>65</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19" t="s">
+        <v>24</v>
+      </c>
+      <c r="O19" t="s">
+        <v>23</v>
+      </c>
+      <c r="P19" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q19" t="b">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <v>0</v>
+      </c>
+      <c r="V19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" t="s">
+        <v>31</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20" t="s">
+        <v>45</v>
+      </c>
+      <c r="I20">
+        <v>7</v>
+      </c>
+      <c r="J20" t="s">
+        <v>22</v>
+      </c>
+      <c r="K20">
+        <v>65</v>
+      </c>
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20" t="s">
+        <v>24</v>
+      </c>
+      <c r="O20" t="s">
+        <v>23</v>
+      </c>
+      <c r="P20" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q20" t="b">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <v>0</v>
+      </c>
+      <c r="V20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21" t="s">
+        <v>45</v>
+      </c>
+      <c r="I21">
+        <v>7</v>
+      </c>
+      <c r="J21" t="s">
+        <v>22</v>
+      </c>
+      <c r="K21">
+        <v>65</v>
+      </c>
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21" t="s">
+        <v>24</v>
+      </c>
+      <c r="O21" t="s">
+        <v>23</v>
+      </c>
+      <c r="P21" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q21" t="b">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <v>0</v>
+      </c>
+      <c r="V21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22" t="s">
+        <v>45</v>
+      </c>
+      <c r="I22">
+        <v>7</v>
+      </c>
+      <c r="J22" t="s">
+        <v>22</v>
+      </c>
+      <c r="K22">
+        <v>65</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22" t="s">
+        <v>24</v>
+      </c>
+      <c r="O22" t="s">
+        <v>23</v>
+      </c>
+      <c r="P22" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q22" t="b">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <v>0</v>
+      </c>
+      <c r="U22">
+        <v>0</v>
+      </c>
+      <c r="V22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" t="s">
+        <v>26</v>
+      </c>
+      <c r="F23" t="s">
+        <v>32</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23" t="s">
+        <v>45</v>
+      </c>
+      <c r="I23">
+        <v>7</v>
+      </c>
+      <c r="J23" t="s">
+        <v>22</v>
+      </c>
+      <c r="K23">
+        <v>65</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23" t="s">
+        <v>24</v>
+      </c>
+      <c r="O23" t="s">
+        <v>23</v>
+      </c>
+      <c r="P23" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q23" t="b">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>0</v>
+      </c>
+      <c r="U23">
+        <v>0</v>
+      </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" t="s">
+        <v>66</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" t="s">
+        <v>26</v>
+      </c>
+      <c r="F24" t="s">
+        <v>32</v>
+      </c>
+      <c r="G24">
+        <v>3</v>
+      </c>
+      <c r="H24" t="s">
+        <v>45</v>
+      </c>
+      <c r="I24">
+        <v>7</v>
+      </c>
+      <c r="J24" t="s">
+        <v>22</v>
+      </c>
+      <c r="K24">
+        <v>65</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24" t="s">
+        <v>24</v>
+      </c>
+      <c r="O24" t="s">
+        <v>23</v>
+      </c>
+      <c r="P24" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q24" t="b">
+        <v>0</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <v>0</v>
+      </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" t="s">
+        <v>66</v>
+      </c>
+      <c r="D25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" t="s">
+        <v>26</v>
+      </c>
+      <c r="F25" t="s">
+        <v>32</v>
+      </c>
+      <c r="G25">
+        <v>4</v>
+      </c>
+      <c r="H25" t="s">
+        <v>45</v>
+      </c>
+      <c r="I25">
+        <v>7</v>
+      </c>
+      <c r="J25" t="s">
+        <v>22</v>
+      </c>
+      <c r="K25">
+        <v>65</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25" t="s">
+        <v>24</v>
+      </c>
+      <c r="O25" t="s">
+        <v>23</v>
+      </c>
+      <c r="P25" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q25" t="b">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>0</v>
+      </c>
+      <c r="U25">
+        <v>0</v>
+      </c>
+      <c r="V25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" t="s">
+        <v>26</v>
+      </c>
+      <c r="F26" t="s">
+        <v>32</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26" t="s">
+        <v>45</v>
+      </c>
+      <c r="I26">
+        <v>7</v>
+      </c>
+      <c r="J26" t="s">
+        <v>22</v>
+      </c>
+      <c r="K26">
+        <v>65</v>
+      </c>
+      <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="N26" t="s">
+        <v>24</v>
+      </c>
+      <c r="O26" t="s">
+        <v>23</v>
+      </c>
+      <c r="P26" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q26" t="b">
+        <v>0</v>
+      </c>
+      <c r="R26">
+        <v>0</v>
+      </c>
+      <c r="S26">
+        <v>0</v>
+      </c>
+      <c r="T26">
+        <v>0</v>
+      </c>
+      <c r="U26">
+        <v>0</v>
+      </c>
+      <c r="V26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" t="s">
+        <v>26</v>
+      </c>
+      <c r="F27" t="s">
+        <v>32</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+      <c r="H27" t="s">
+        <v>45</v>
+      </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
+      <c r="J27" t="s">
+        <v>22</v>
+      </c>
+      <c r="K27">
+        <v>65</v>
+      </c>
+      <c r="M27">
+        <v>0</v>
+      </c>
+      <c r="N27" t="s">
+        <v>24</v>
+      </c>
+      <c r="O27" t="s">
+        <v>23</v>
+      </c>
+      <c r="P27" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q27" t="b">
+        <v>0</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+      <c r="S27">
+        <v>0</v>
+      </c>
+      <c r="T27">
+        <v>0</v>
+      </c>
+      <c r="U27">
+        <v>0</v>
+      </c>
+      <c r="V27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" t="s">
+        <v>32</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28" t="s">
+        <v>45</v>
+      </c>
+      <c r="I28">
+        <v>7</v>
+      </c>
+      <c r="J28" t="s">
+        <v>22</v>
+      </c>
+      <c r="K28">
+        <v>65</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28" t="s">
+        <v>24</v>
+      </c>
+      <c r="O28" t="s">
+        <v>23</v>
+      </c>
+      <c r="P28" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q28" t="b">
+        <v>0</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+      <c r="S28">
+        <v>0</v>
+      </c>
+      <c r="T28">
+        <v>0</v>
+      </c>
+      <c r="U28">
+        <v>0</v>
+      </c>
+      <c r="V28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>32</v>
+      </c>
+      <c r="G29">
+        <v>2</v>
+      </c>
+      <c r="H29" t="s">
+        <v>45</v>
+      </c>
+      <c r="I29">
+        <v>7</v>
+      </c>
+      <c r="J29" t="s">
+        <v>22</v>
+      </c>
+      <c r="K29">
+        <v>65</v>
+      </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29" t="s">
+        <v>24</v>
+      </c>
+      <c r="O29" t="s">
+        <v>23</v>
+      </c>
+      <c r="P29" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q29" t="b">
+        <v>0</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+      <c r="S29">
+        <v>0</v>
+      </c>
+      <c r="T29">
+        <v>0</v>
+      </c>
+      <c r="U29">
+        <v>0</v>
+      </c>
+      <c r="V29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30" t="s">
+        <v>72</v>
+      </c>
+      <c r="E30" t="s">
+        <v>35</v>
+      </c>
+      <c r="F30" t="s">
+        <v>38</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30" t="s">
+        <v>45</v>
+      </c>
+      <c r="I30">
+        <v>7</v>
+      </c>
+      <c r="J30" t="s">
+        <v>34</v>
+      </c>
+      <c r="K30">
+        <v>65</v>
+      </c>
+      <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30" t="s">
+        <v>24</v>
+      </c>
+      <c r="O30" t="s">
+        <v>23</v>
+      </c>
+      <c r="P30" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q30" t="b">
+        <v>0</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30">
+        <v>0</v>
+      </c>
+      <c r="U30">
+        <v>0</v>
+      </c>
+      <c r="V30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" t="s">
+        <v>71</v>
+      </c>
+      <c r="D31" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" t="s">
+        <v>35</v>
+      </c>
+      <c r="F31" t="s">
+        <v>38</v>
+      </c>
+      <c r="G31">
+        <v>2</v>
+      </c>
+      <c r="H31" t="s">
+        <v>45</v>
+      </c>
+      <c r="I31">
+        <v>7</v>
+      </c>
+      <c r="J31" t="s">
+        <v>34</v>
+      </c>
+      <c r="K31">
+        <v>65</v>
+      </c>
+      <c r="M31">
+        <v>0</v>
+      </c>
+      <c r="N31" t="s">
+        <v>24</v>
+      </c>
+      <c r="O31" t="s">
+        <v>23</v>
+      </c>
+      <c r="P31" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q31" t="b">
+        <v>0</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>0</v>
+      </c>
+      <c r="U31">
+        <v>0</v>
+      </c>
+      <c r="V31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" t="s">
+        <v>35</v>
+      </c>
+      <c r="F32" t="s">
+        <v>38</v>
+      </c>
+      <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32" t="s">
+        <v>45</v>
+      </c>
+      <c r="I32">
+        <v>7</v>
+      </c>
+      <c r="J32" t="s">
+        <v>34</v>
+      </c>
+      <c r="K32">
+        <v>65</v>
+      </c>
+      <c r="M32">
+        <v>0</v>
+      </c>
+      <c r="N32" t="s">
+        <v>24</v>
+      </c>
+      <c r="O32" t="s">
+        <v>23</v>
+      </c>
+      <c r="P32" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="S32">
+        <v>0</v>
+      </c>
+      <c r="T32">
+        <v>0</v>
+      </c>
+      <c r="U32">
+        <v>0</v>
+      </c>
+      <c r="V32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" t="s">
+        <v>71</v>
+      </c>
+      <c r="D33" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33" t="s">
+        <v>35</v>
+      </c>
+      <c r="F33" t="s">
+        <v>38</v>
+      </c>
+      <c r="G33">
+        <v>2</v>
+      </c>
+      <c r="H33" t="s">
+        <v>45</v>
+      </c>
+      <c r="I33">
+        <v>7</v>
+      </c>
+      <c r="J33" t="s">
+        <v>34</v>
+      </c>
+      <c r="K33">
+        <v>65</v>
+      </c>
+      <c r="M33">
+        <v>0</v>
+      </c>
+      <c r="N33" t="s">
+        <v>24</v>
+      </c>
+      <c r="O33" t="s">
+        <v>23</v>
+      </c>
+      <c r="P33" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q33" t="b">
+        <v>0</v>
+      </c>
+      <c r="R33">
+        <v>0</v>
+      </c>
+      <c r="S33">
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <v>0</v>
+      </c>
+      <c r="U33">
+        <v>0</v>
+      </c>
+      <c r="V33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>75</v>
+      </c>
+      <c r="B34" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" t="s">
+        <v>39</v>
+      </c>
+      <c r="E34" t="s">
+        <v>35</v>
+      </c>
+      <c r="F34" t="s">
+        <v>38</v>
+      </c>
+      <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34" t="s">
+        <v>45</v>
+      </c>
+      <c r="I34">
+        <v>7</v>
+      </c>
+      <c r="J34" t="s">
+        <v>34</v>
+      </c>
+      <c r="K34">
+        <v>65</v>
+      </c>
+      <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34" t="s">
+        <v>24</v>
+      </c>
+      <c r="O34" t="s">
+        <v>23</v>
+      </c>
+      <c r="P34" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q34" t="b">
+        <v>0</v>
+      </c>
+      <c r="R34">
+        <v>0</v>
+      </c>
+      <c r="S34">
+        <v>0</v>
+      </c>
+      <c r="T34">
+        <v>0</v>
+      </c>
+      <c r="U34">
+        <v>0</v>
+      </c>
+      <c r="V34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>75</v>
+      </c>
+      <c r="B35" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" t="s">
+        <v>39</v>
+      </c>
+      <c r="E35" t="s">
+        <v>35</v>
+      </c>
+      <c r="F35" t="s">
+        <v>38</v>
+      </c>
+      <c r="G35">
+        <v>2</v>
+      </c>
+      <c r="H35" t="s">
+        <v>45</v>
+      </c>
+      <c r="I35">
+        <v>7</v>
+      </c>
+      <c r="J35" t="s">
+        <v>34</v>
+      </c>
+      <c r="K35">
+        <v>65</v>
+      </c>
+      <c r="M35">
+        <v>0</v>
+      </c>
+      <c r="N35" t="s">
+        <v>24</v>
+      </c>
+      <c r="O35" t="s">
+        <v>23</v>
+      </c>
+      <c r="P35" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q35" t="b">
+        <v>0</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+      <c r="S35">
+        <v>0</v>
+      </c>
+      <c r="T35">
+        <v>0</v>
+      </c>
+      <c r="U35">
+        <v>0</v>
+      </c>
+      <c r="V35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" t="s">
+        <v>39</v>
+      </c>
+      <c r="E36" t="s">
+        <v>35</v>
+      </c>
+      <c r="F36" t="s">
+        <v>38</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36" t="s">
+        <v>45</v>
+      </c>
+      <c r="I36">
+        <v>7</v>
+      </c>
+      <c r="J36" t="s">
+        <v>34</v>
+      </c>
+      <c r="K36">
+        <v>65</v>
+      </c>
+      <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36" t="s">
+        <v>24</v>
+      </c>
+      <c r="O36" t="s">
+        <v>23</v>
+      </c>
+      <c r="P36" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R36">
+        <v>0</v>
+      </c>
+      <c r="S36">
+        <v>0</v>
+      </c>
+      <c r="T36">
+        <v>0</v>
+      </c>
+      <c r="U36">
+        <v>0</v>
+      </c>
+      <c r="V36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" t="s">
+        <v>39</v>
+      </c>
+      <c r="E37" t="s">
+        <v>35</v>
+      </c>
+      <c r="F37" t="s">
+        <v>38</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+      <c r="H37" t="s">
+        <v>45</v>
+      </c>
+      <c r="I37">
+        <v>7</v>
+      </c>
+      <c r="J37" t="s">
+        <v>34</v>
+      </c>
+      <c r="K37">
+        <v>65</v>
+      </c>
+      <c r="M37">
+        <v>0</v>
+      </c>
+      <c r="N37" t="s">
+        <v>24</v>
+      </c>
+      <c r="O37" t="s">
+        <v>23</v>
+      </c>
+      <c r="P37" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q37" t="b">
+        <v>0</v>
+      </c>
+      <c r="R37">
+        <v>0</v>
+      </c>
+      <c r="S37">
+        <v>0</v>
+      </c>
+      <c r="T37">
+        <v>0</v>
+      </c>
+      <c r="U37">
+        <v>0</v>
+      </c>
+      <c r="V37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" t="s">
+        <v>33</v>
+      </c>
+      <c r="D38" t="s">
+        <v>28</v>
+      </c>
+      <c r="E38" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38" t="s">
+        <v>30</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38" t="s">
+        <v>45</v>
+      </c>
+      <c r="I38">
+        <v>7</v>
+      </c>
+      <c r="J38" t="s">
+        <v>22</v>
+      </c>
+      <c r="K38">
+        <v>65</v>
+      </c>
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38" t="s">
+        <v>24</v>
+      </c>
+      <c r="O38" t="s">
+        <v>23</v>
+      </c>
+      <c r="P38" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q38" t="b">
+        <v>0</v>
+      </c>
+      <c r="R38">
+        <v>0</v>
+      </c>
+      <c r="S38">
+        <v>0</v>
+      </c>
+      <c r="T38">
+        <v>0</v>
+      </c>
+      <c r="U38">
+        <v>0</v>
+      </c>
+      <c r="V38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>80</v>
+      </c>
+      <c r="B39" t="s">
+        <v>33</v>
+      </c>
+      <c r="D39" t="s">
+        <v>28</v>
+      </c>
+      <c r="E39" t="s">
+        <v>29</v>
+      </c>
+      <c r="F39" t="s">
+        <v>30</v>
+      </c>
+      <c r="G39">
+        <v>2</v>
+      </c>
+      <c r="H39" t="s">
+        <v>45</v>
+      </c>
+      <c r="I39">
+        <v>7</v>
+      </c>
+      <c r="J39" t="s">
+        <v>22</v>
+      </c>
+      <c r="K39">
+        <v>65</v>
+      </c>
+      <c r="M39">
+        <v>0</v>
+      </c>
+      <c r="N39" t="s">
+        <v>24</v>
+      </c>
+      <c r="O39" t="s">
+        <v>23</v>
+      </c>
+      <c r="P39" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q39" t="b">
+        <v>0</v>
+      </c>
+      <c r="R39">
+        <v>0</v>
+      </c>
+      <c r="S39">
+        <v>0</v>
+      </c>
+      <c r="T39">
+        <v>0</v>
+      </c>
+      <c r="U39">
+        <v>0</v>
+      </c>
+      <c r="V39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" t="s">
+        <v>36</v>
+      </c>
+      <c r="D40" t="s">
+        <v>28</v>
+      </c>
+      <c r="E40" t="s">
+        <v>29</v>
+      </c>
+      <c r="F40" t="s">
         <v>37</v>
       </c>
-      <c r="Q17" t="b">
-        <v>0</v>
-      </c>
-      <c r="R17">
-        <v>0</v>
-      </c>
-      <c r="S17">
-        <v>0</v>
-      </c>
-      <c r="T17">
-        <v>0</v>
-      </c>
-      <c r="U17">
-        <v>0</v>
-      </c>
-      <c r="V17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H31" s="2"/>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H32" s="2"/>
-    </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H33" s="2"/>
-    </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H35" s="2"/>
-    </row>
-    <row r="36" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H37" s="2"/>
-    </row>
-    <row r="38" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H38" s="2"/>
-    </row>
-    <row r="39" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H39" s="2"/>
-    </row>
-    <row r="40" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H40" s="2"/>
-    </row>
-    <row r="41" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H41" s="2"/>
-    </row>
-    <row r="42" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H42" s="2"/>
-    </row>
-    <row r="43" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H43" s="2"/>
-    </row>
-    <row r="44" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H44" s="2"/>
-    </row>
-    <row r="45" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H45" s="2"/>
-    </row>
-    <row r="46" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H46" s="2"/>
-    </row>
-    <row r="47" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H47" s="2"/>
-    </row>
-    <row r="48" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H48" s="2"/>
-    </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H49" s="2"/>
-    </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H50" s="2"/>
-    </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H51" s="2"/>
-    </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H52" s="2"/>
-    </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H53" s="2"/>
-    </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H54" s="2"/>
-    </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H55" s="2"/>
-    </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H56" s="2"/>
-    </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H57" s="2"/>
-    </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H58" s="2"/>
-    </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H59" s="2"/>
-    </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H60" s="2"/>
-    </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H61" s="2"/>
-    </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H62" s="2"/>
-    </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H63" s="2"/>
-    </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H64" s="2"/>
-    </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H65" s="2"/>
-    </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H66" s="2"/>
-    </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H67" s="2"/>
-    </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H68" s="2"/>
-    </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H69" s="2"/>
-    </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H70" s="2"/>
-    </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H71" s="2"/>
-    </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H72" s="2"/>
-    </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H73" s="2"/>
-    </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H74" s="2"/>
-    </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H75" s="2"/>
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40" t="s">
+        <v>45</v>
+      </c>
+      <c r="I40">
+        <v>7</v>
+      </c>
+      <c r="J40" t="s">
+        <v>22</v>
+      </c>
+      <c r="K40">
+        <v>65</v>
+      </c>
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40" t="s">
+        <v>24</v>
+      </c>
+      <c r="O40" t="s">
+        <v>23</v>
+      </c>
+      <c r="P40" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q40" t="b">
+        <v>0</v>
+      </c>
+      <c r="R40">
+        <v>0</v>
+      </c>
+      <c r="S40">
+        <v>0</v>
+      </c>
+      <c r="T40">
+        <v>0</v>
+      </c>
+      <c r="U40">
+        <v>0</v>
+      </c>
+      <c r="V40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" t="s">
+        <v>36</v>
+      </c>
+      <c r="D41" t="s">
+        <v>28</v>
+      </c>
+      <c r="E41" t="s">
+        <v>29</v>
+      </c>
+      <c r="F41" t="s">
+        <v>37</v>
+      </c>
+      <c r="G41">
+        <v>2</v>
+      </c>
+      <c r="H41" t="s">
+        <v>45</v>
+      </c>
+      <c r="I41">
+        <v>7</v>
+      </c>
+      <c r="J41" t="s">
+        <v>22</v>
+      </c>
+      <c r="K41">
+        <v>65</v>
+      </c>
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41" t="s">
+        <v>24</v>
+      </c>
+      <c r="O41" t="s">
+        <v>23</v>
+      </c>
+      <c r="P41" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q41" t="b">
+        <v>0</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
+      </c>
+      <c r="S41">
+        <v>0</v>
+      </c>
+      <c r="T41">
+        <v>0</v>
+      </c>
+      <c r="U41">
+        <v>0</v>
+      </c>
+      <c r="V41">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AD1" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>